<commit_message>
bug fix with gear list
when not all attribution were listed, the code wouldn't work.
</commit_message>
<xml_diff>
--- a/3f_v0_test.xlsx
+++ b/3f_v0_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hmgenet\Downloads\3F-main\3F-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA37E5C-73BC-4CCF-8423-AA0DB1D5AE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856174A0-B9FC-4C43-B87D-98FF0E634709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1665" windowWidth="29040" windowHeight="15720" tabRatio="944" activeTab="1" xr2:uid="{19575149-6688-42F2-88E3-84A9785EF7E3}"/>
+    <workbookView xWindow="28680" yWindow="1665" windowWidth="29040" windowHeight="15720" tabRatio="944" activeTab="2" xr2:uid="{19575149-6688-42F2-88E3-84A9785EF7E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Flight_inventory" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -329,7 +329,7 @@
 inputs['Heli manager'] = inputs['Heli manager'].fillna("")
 inputs['Going to the plot?'] = inputs['Going to the plot?'].fillna("")
 inputs['Hazardous materials'] = inputs['Hazardous materials'].fillna("")
-inputs['Extra weight (lbs)?'] = inputs['Extra weight (lbs)?'].fillna("")
+inputs['Extra weight (lbs)?'] = inputs['Extra weight (lbs)?'].fillna(0)
 ndfl = pd.DataFrame(inputs.groupby(['Date', 'Hub', 'Flight number', 'Pilot', 'Heli manager','Going to the plot?','Hazardous materials'])['Drop off'].count())
 ndfl.reset_index(inplace=True)
 ndfl = ndfl.rename(columns={'Drop off':'ndf'})
@@ -431,7 +431,13 @@
 		else:
 			m = 0
 		wlist.append(m)
-	wgear = (len(lcf) * gears_sum[gears_sum['Attribution'] == 'per passenger']['totweight'].values) + (ndo * gears_sum[gears_sum['Attribution'] == 'per drop-off']['totweight'].values) + gears_sum[gears_sum['Attribution'] == 'per flight']['totweight'].values
+	wgear=inputs[inputs['Flight number'] == float(listfn[i].removeprefix("Flight "))]['Extra weight (lbs)?'].sum()
+	if 'per passenger' in gears_sum['Attribution'].tolist():
+		wgear += (len(lcf) * gears_sum[gears_sum['Attribution'] == 'per passenger']['totweight'].values) 
+	if 'per drop-off' in 	gears_sum['Attribution'].tolist():
+		wgear += (ndo * gears_sum[gears_sum['Attribution'] == 'per drop-off']['totweight'].values) 
+	if 'per flight' in 	gears_sum['Attribution'].tolist():
+		wgear += gears_sum[gears_sum['Attribution'] == 'per flight']['totweight'].values
 	wgt = [""]
 	for j in range(nr):
 		if j == 1:
@@ -458,6 +464,7 @@
 		else:
 			result.append(item)
 	listweight = listweight + result
+	listweight
 np.column_stack((listflt, listdescr, listweight))
 </code>
     </pythonScript>
@@ -466,7 +473,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="79">
   <si>
     <t>Flight number</t>
   </si>
@@ -748,6 +755,9 @@
   </si>
   <si>
     <t>elevation (ft)</t>
+  </si>
+  <si>
+    <t>ammo</t>
   </si>
 </sst>
 </file>
@@ -2471,7 +2481,9 @@
       <c r="F7" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="110"/>
+      <c r="G7" s="110" t="s">
+        <v>78</v>
+      </c>
       <c r="H7" s="40">
         <v>1</v>
       </c>
@@ -4216,6 +4228,7 @@
       <c r="Q51" s="51"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="UtP+XElkmSvOs4jF4MVAsMZkvO8d9HaeydYNyyFpbVwWR6zGCZlQcUzYqz3cKba1tBOLM8olmVGgSltq19ABng==" saltValue="1vKxb8c5g/Z1BfKv5aTW1A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -4613,6 +4626,7 @@
       <c r="D41" s="70"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="WYUuzb7ZMmcfke3EfOzTEy1p31qqu4WE1Rts7u2ADrVot+0d0ek5Uq8fFCLCZaxz8jglXhpVi9JPaqSau0rPfA==" saltValue="wxADVolFzLyMrbB3u6FNVA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C41" xr:uid="{F443EC5B-F211-4329-983E-60BD86B9E5D3}">
       <formula1>$H$2:$H$4</formula1>
@@ -6530,6 +6544,7 @@
       <c r="J173" s="7"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="b8Y3IYSkI8r65S3qQzXtfdkBI4yPpNV6AzHhAIFBwFBq0cOebdRJ4u6HXbbjNFADG5UVqWwWfyqasZCLiuZt2A==" saltValue="QqMGuintGpCFp+gYanNl/A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -6652,7 +6667,7 @@
         <v>standard gear list + extra weight</v>
       </c>
       <c r="C10" s="62" t="str">
-        <v>2220.0</v>
+        <v>2280.0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -6685,7 +6700,7 @@
         <v/>
       </c>
       <c r="C13" s="68" t="str">
-        <v>3000.0</v>
+        <v>3060.0</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="69" customFormat="1" x14ac:dyDescent="0.3">
@@ -6836,7 +6851,7 @@
         <v>Hazardous materials:</v>
       </c>
       <c r="B27" s="69" t="str">
-        <v/>
+        <v>ammo</v>
       </c>
       <c r="C27" s="69" t="str">
         <v/>
@@ -7262,6 +7277,7 @@
       <c r="C131" s="69"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="CMNcugR6T7R1XGxe8URRpoFZAQS6thnbdIa6mqp4L9ufuvA4TutkF+aid0xHPe0J5W3vqBbtR9REepcginAXjQ==" saltValue="DBLMdgIHJ7HD+lNyJN3WqA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>

</xml_diff>